<commit_message>
Lĩnh vực: 11 nhóm ngành cố định
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GIAO-THUONG-DATA.xlsx
+++ b/GIAO-THUONG-DATA.xlsx
@@ -2,36 +2,191 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="27660" windowHeight="11740" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="TinDang" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="KetNoi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="NhomNganh" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
+  <fonts count="22">
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -40,11 +195,198 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001565D8"/>
+        <fgColor rgb="FF1565D8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -52,17 +394,307 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="49">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -415,7 +1047,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -426,23 +1057,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8" outlineLevelRow="4"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="13.796875" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -550,7 +1168,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Truyền thông - Sự kiện</t>
+          <t>Truyền thông sự kiện - nghiên cứu thị trường</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -571,6 +1189,11 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>duyet</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Truyền thông sự kiện - nghiên cứu thị trường</t>
         </is>
       </c>
     </row>
@@ -602,7 +1225,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Điện - Điện tử - Điện lạnh</t>
+          <t>Tổng thầu cơ điện công trình (M&amp;E) và lắp đặt hệ thống</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -623,6 +1246,11 @@
       <c r="K3" t="inlineStr">
         <is>
           <t>duyet</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Tổng thầu cơ điện công trình (M&amp;E) và lắp đặt hệ thống</t>
         </is>
       </c>
     </row>
@@ -654,7 +1282,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Cơ khí - Chế tạo</t>
+          <t>Gia công cơ khí chính xác</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -716,7 +1344,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Khác</t>
+          <t>Cơ khí chế tạo máy</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -739,14 +1367,22 @@
           <t>cho_duyet</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Cơ khí chế tạo máy</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="A2:A1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"mua,ban"</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"duyet,cho_duyet,an"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>=NhomNganh!$B$2:$B$12</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -760,23 +1396,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="1" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -854,4 +1476,143 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="70" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>so</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>nhom_nganh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cơ khí chế tạo máy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Gia công cơ khí chính xác</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Khuôn mẫu và Công nghiệp hỗ trợ (CNHT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kết cấu thép</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sản xuất thiết bị điện - điều khiển - tự động hoá - công nghệ số</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tổng thầu cơ điện công trình (M&amp;E) và lắp đặt hệ thống</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Thiết bị và giải pháp năng lượng – môi trường</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ngành nông lâm thuỷ hải sản LTTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ngành cao su nhựa</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ngành chế biến gỗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Truyền thông sự kiện - nghiên cứu thị trường</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Group industries: cơ khí–điện vs ngành phục vụ
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GIAO-THUONG-DATA.xlsx
+++ b/GIAO-THUONG-DATA.xlsx
@@ -1484,10 +1484,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1501,6 +1502,11 @@
           <t>nhom_nganh</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>cum</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1511,6 +1517,11 @@
           <t>Cơ khí chế tạo máy</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Chuyên ngành cơ khí – điện</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1521,6 +1532,11 @@
           <t>Gia công cơ khí chính xác</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Chuyên ngành cơ khí – điện</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1531,6 +1547,11 @@
           <t>Khuôn mẫu và Công nghiệp hỗ trợ (CNHT)</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Chuyên ngành cơ khí – điện</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1541,6 +1562,11 @@
           <t>Kết cấu thép</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Chuyên ngành cơ khí – điện</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1551,6 +1577,11 @@
           <t>Sản xuất thiết bị điện - điều khiển - tự động hoá - công nghệ số</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Chuyên ngành cơ khí – điện</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1561,6 +1592,11 @@
           <t>Tổng thầu cơ điện công trình (M&amp;E) và lắp đặt hệ thống</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Chuyên ngành cơ khí – điện</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1571,6 +1607,11 @@
           <t>Thiết bị và giải pháp năng lượng – môi trường</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Chuyên ngành cơ khí – điện</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1581,6 +1622,11 @@
           <t>Ngành nông lâm thuỷ hải sản LTTP</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Ngành phục vụ</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1591,6 +1637,11 @@
           <t>Ngành cao su nhựa</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ngành phục vụ</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1601,6 +1652,11 @@
           <t>Ngành chế biến gỗ</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ngành phục vụ</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1609,6 +1665,11 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>Truyền thông sự kiện - nghiên cứu thị trường</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ngành phục vụ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ngành nghề: 6 nhóm
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GIAO-THUONG-DATA.xlsx
+++ b/GIAO-THUONG-DATA.xlsx
@@ -1168,7 +1168,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Truyền thông sự kiện - nghiên cứu thị trường</t>
+          <t>Nhóm truyền thông - sự kiện - nghiên cứu</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Truyền thông sự kiện - nghiên cứu thị trường</t>
+          <t>Nhóm truyền thông - sự kiện - nghiên cứu</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Tổng thầu cơ điện công trình (M&amp;E) và lắp đặt hệ thống</t>
+          <t>Nhóm ngành cơ khí - điện</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Tổng thầu cơ điện công trình (M&amp;E) và lắp đặt hệ thống</t>
+          <t>Nhóm ngành cơ khí - điện</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Gia công cơ khí chính xác</t>
+          <t>Nhóm ngành cơ khí - điện</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Gia công cơ khí chính xác</t>
+          <t>Nhóm ngành cơ khí - điện</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Cơ khí chế tạo máy</t>
+          <t>Nhóm ngành cơ khí - điện</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Cơ khí chế tạo máy</t>
+          <t>Nhóm ngành cơ khí - điện</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
       <formula1>"duyet,cho_duyet,an"</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=NhomNganh!$B$2:$B$12</formula1>
+      <formula1>=NhomNganh!$B$2:$B$7</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1484,11 +1484,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1502,11 +1501,6 @@
           <t>nhom_nganh</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>cum</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1514,12 +1508,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cơ khí chế tạo máy</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Chuyên ngành cơ khí – điện</t>
+          <t>Nhóm truyền thông - sự kiện - nghiên cứu</t>
         </is>
       </c>
     </row>
@@ -1529,12 +1518,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Gia công cơ khí chính xác</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Chuyên ngành cơ khí – điện</t>
+          <t>Nhóm ngành cơ khí - điện</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1528,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Khuôn mẫu và Công nghiệp hỗ trợ (CNHT)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Chuyên ngành cơ khí – điện</t>
+          <t>Nhóm ngành xây dựng</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1538,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kết cấu thép</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Chuyên ngành cơ khí – điện</t>
+          <t>Nhóm ngành chế biến gỗ</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1548,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sản xuất thiết bị điện - điều khiển - tự động hoá - công nghệ số</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Chuyên ngành cơ khí – điện</t>
+          <t>Nhóm ngành cao su nhựa</t>
         </is>
       </c>
     </row>
@@ -1589,87 +1558,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tổng thầu cơ điện công trình (M&amp;E) và lắp đặt hệ thống</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Chuyên ngành cơ khí – điện</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Thiết bị và giải pháp năng lượng – môi trường</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Chuyên ngành cơ khí – điện</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Ngành nông lâm thuỷ hải sản LTTP</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Ngành phục vụ</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Ngành cao su nhựa</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Ngành phục vụ</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Ngành chế biến gỗ</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Ngành phục vụ</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Truyền thông sự kiện - nghiên cứu thị trường</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Ngành phục vụ</t>
+          <t>Nông lâm thuỷ hải sản</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Thêm nhóm vận tải-logistics, điện tử-bán dẫn
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GIAO-THUONG-DATA.xlsx
+++ b/GIAO-THUONG-DATA.xlsx
@@ -1382,7 +1382,7 @@
       <formula1>"duyet,cho_duyet,an"</formula1>
     </dataValidation>
     <dataValidation sqref="N2:N1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=NhomNganh!$B$2:$B$7</formula1>
+      <formula1>=NhomNganh!$B$2:$B$9</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1484,7 +1484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="2" max="2"/>
@@ -1562,6 +1562,26 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Nhóm ngành vận tải - logistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Nhóm ngành điện tử - bán dẫn</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ngành nghề: 8 nhóm theo HAMEE
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GIAO-THUONG-DATA.xlsx
+++ b/GIAO-THUONG-DATA.xlsx
@@ -1168,7 +1168,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Nhóm truyền thông - sự kiện - nghiên cứu</t>
+          <t>Truyền thông - nghiên cứu</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Nhóm truyền thông - sự kiện - nghiên cứu</t>
+          <t>Truyền thông - nghiên cứu</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Nhóm ngành cơ khí - điện</t>
+          <t>Cơ khí - điện - năng lượng</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Nhóm ngành cơ khí - điện</t>
+          <t>Cơ khí - điện - năng lượng</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Nhóm ngành cơ khí - điện</t>
+          <t>Cơ khí - điện - năng lượng</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Nhóm ngành cơ khí - điện</t>
+          <t>Cơ khí - điện - năng lượng</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Nhóm ngành cơ khí - điện</t>
+          <t>Cơ khí - điện - năng lượng</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Nhóm ngành cơ khí - điện</t>
+          <t>Cơ khí - điện - năng lượng</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nhóm truyền thông - sự kiện - nghiên cứu</t>
+          <t>Cơ khí - điện - năng lượng</t>
         </is>
       </c>
     </row>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nhóm ngành cơ khí - điện</t>
+          <t>Tự động hoá - công nghệ số</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nhóm ngành xây dựng</t>
+          <t>Vận tải - logistics</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nhóm ngành chế biến gỗ</t>
+          <t>Xây dựng</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nhóm ngành cao su nhựa</t>
+          <t>Cao su nhựa</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Nông lâm thuỷ hải sản</t>
+          <t>Chế biến gỗ</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nhóm ngành vận tải - logistics</t>
+          <t>Nông lâm thuỷ hải sản</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Nhóm ngành điện tử - bán dẫn</t>
+          <t>Truyền thông - nghiên cứu</t>
         </is>
       </c>
     </row>

</xml_diff>